<commit_message>
Hogar de Refugio: canaleta de las 9 bancas OC-01 (3 juegos) en RESUMEN, PLANILLA y hoja propia del metrado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_CANALETA_OC-01_BANCA_PERGOLA_HOGAR_REFUGIO.xlsx
+++ b/entregables/METRADO_CANALETA_OC-01_BANCA_PERGOLA_HOGAR_REFUGIO.xlsx
@@ -591,11 +591,11 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>N.° DE ESTRUCTURAS OC-01</t>
+          <t>N.° DE JUEGOS OC-01 (9 BANCAS)</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">

</xml_diff>